<commit_message>
Backup 2026-10: Firestore-Stand + Excel-Auswertung
</commit_message>
<xml_diff>
--- a/backup/2026-10_kataster.xlsx
+++ b/backup/2026-10_kataster.xlsx
@@ -4111,7 +4111,11 @@
       </c>
       <c r="D63" t="inlineStr"/>
       <c r="E63" t="inlineStr"/>
-      <c r="F63" t="inlineStr"/>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
       <c r="G63" t="inlineStr"/>
       <c r="H63" t="inlineStr">
         <is>
@@ -4154,7 +4158,11 @@
       </c>
       <c r="D64" t="inlineStr"/>
       <c r="E64" t="inlineStr"/>
-      <c r="F64" t="inlineStr"/>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
       <c r="G64" t="inlineStr"/>
       <c r="H64" t="inlineStr">
         <is>
@@ -4197,7 +4205,11 @@
       </c>
       <c r="D65" t="inlineStr"/>
       <c r="E65" t="inlineStr"/>
-      <c r="F65" t="inlineStr"/>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
       <c r="G65" t="inlineStr"/>
       <c r="H65" t="inlineStr">
         <is>
@@ -4240,7 +4252,11 @@
       </c>
       <c r="D66" t="inlineStr"/>
       <c r="E66" t="inlineStr"/>
-      <c r="F66" t="inlineStr"/>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
       <c r="G66" t="inlineStr">
         <is>
           <t>Walnussreihe (Einzelposition im Lageplan noch offen)</t>
@@ -4287,7 +4303,11 @@
       </c>
       <c r="D67" t="inlineStr"/>
       <c r="E67" t="inlineStr"/>
-      <c r="F67" t="inlineStr"/>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
       <c r="G67" t="inlineStr"/>
       <c r="H67" t="inlineStr">
         <is>
@@ -4330,7 +4350,11 @@
       </c>
       <c r="D68" t="inlineStr"/>
       <c r="E68" t="inlineStr"/>
-      <c r="F68" t="inlineStr"/>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
       <c r="G68" t="inlineStr"/>
       <c r="H68" t="inlineStr">
         <is>
@@ -4373,7 +4397,11 @@
       </c>
       <c r="D69" t="inlineStr"/>
       <c r="E69" t="inlineStr"/>
-      <c r="F69" t="inlineStr"/>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
       <c r="G69" t="inlineStr"/>
       <c r="H69" t="inlineStr">
         <is>
@@ -4416,7 +4444,11 @@
       </c>
       <c r="D70" t="inlineStr"/>
       <c r="E70" t="inlineStr"/>
-      <c r="F70" t="inlineStr"/>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
       <c r="G70" t="inlineStr"/>
       <c r="H70" t="inlineStr">
         <is>
@@ -4459,7 +4491,11 @@
       </c>
       <c r="D71" t="inlineStr"/>
       <c r="E71" t="inlineStr"/>
-      <c r="F71" t="inlineStr"/>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
       <c r="G71" t="inlineStr"/>
       <c r="H71" t="inlineStr">
         <is>
@@ -4502,7 +4538,11 @@
       </c>
       <c r="D72" t="inlineStr"/>
       <c r="E72" t="inlineStr"/>
-      <c r="F72" t="inlineStr"/>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
       <c r="G72" t="inlineStr"/>
       <c r="H72" t="inlineStr">
         <is>
@@ -4545,7 +4585,11 @@
       </c>
       <c r="D73" t="inlineStr"/>
       <c r="E73" t="inlineStr"/>
-      <c r="F73" t="inlineStr"/>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
       <c r="G73" t="inlineStr"/>
       <c r="H73" t="inlineStr">
         <is>
@@ -4588,7 +4632,11 @@
       </c>
       <c r="D74" t="inlineStr"/>
       <c r="E74" t="inlineStr"/>
-      <c r="F74" t="inlineStr"/>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
       <c r="G74" t="inlineStr"/>
       <c r="H74" t="inlineStr">
         <is>
@@ -4631,7 +4679,11 @@
       </c>
       <c r="D75" t="inlineStr"/>
       <c r="E75" t="inlineStr"/>
-      <c r="F75" t="inlineStr"/>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
       <c r="G75" t="inlineStr"/>
       <c r="H75" t="inlineStr">
         <is>
@@ -4674,7 +4726,11 @@
       </c>
       <c r="D76" t="inlineStr"/>
       <c r="E76" t="inlineStr"/>
-      <c r="F76" t="inlineStr"/>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
       <c r="G76" t="inlineStr"/>
       <c r="H76" t="inlineStr">
         <is>
@@ -4717,7 +4773,11 @@
       </c>
       <c r="D77" t="inlineStr"/>
       <c r="E77" t="inlineStr"/>
-      <c r="F77" t="inlineStr"/>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
       <c r="G77" t="inlineStr"/>
       <c r="H77" t="inlineStr">
         <is>
@@ -4760,7 +4820,11 @@
       </c>
       <c r="D78" t="inlineStr"/>
       <c r="E78" t="inlineStr"/>
-      <c r="F78" t="inlineStr"/>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
       <c r="G78" t="inlineStr"/>
       <c r="H78" t="inlineStr">
         <is>
@@ -4803,7 +4867,11 @@
       </c>
       <c r="D79" t="inlineStr"/>
       <c r="E79" t="inlineStr"/>
-      <c r="F79" t="inlineStr"/>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
       <c r="G79" t="inlineStr"/>
       <c r="H79" t="inlineStr">
         <is>
@@ -4846,7 +4914,11 @@
       </c>
       <c r="D80" t="inlineStr"/>
       <c r="E80" t="inlineStr"/>
-      <c r="F80" t="inlineStr"/>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
       <c r="G80" t="inlineStr"/>
       <c r="H80" t="inlineStr">
         <is>
@@ -4889,7 +4961,11 @@
       </c>
       <c r="D81" t="inlineStr"/>
       <c r="E81" t="inlineStr"/>
-      <c r="F81" t="inlineStr"/>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
       <c r="G81" t="inlineStr"/>
       <c r="H81" t="inlineStr">
         <is>
@@ -4932,7 +5008,11 @@
       </c>
       <c r="D82" t="inlineStr"/>
       <c r="E82" t="inlineStr"/>
-      <c r="F82" t="inlineStr"/>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
       <c r="G82" t="inlineStr"/>
       <c r="H82" t="inlineStr"/>
       <c r="I82" t="inlineStr"/>

</xml_diff>